<commit_message>
Group live search lot details columns
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -398,7 +398,7 @@
     <t>MSTC LIMITED  •  LIVE SEARCH   (results grouped by the value you typed, each group totalled, TOTAL MATCHED beneath them, the misses greyed in a REMAINING block, a GRAND TOTAL of both at the foot)</t>
   </si>
   <si>
-    <t>HOW TO USE  ▶  click the yellow box B3 and type - a lot number (1874), part of one (187), a buyer (NATIONAL), part of a buyer name, a lot name (COPPER).   •   WILDCARD / MATCH ANY - separate values with a comma or a slash:   1874, 1923, OMKAR   or   1874 / 1923    - and every lot containing ANY of them lights up.   •   COLUMN SEARCHES - type above any column header in row 4; comma or slash means ANY value in that column, * matches any text and ? matches one character.  Filters entered in different columns are combined as ALL.   •   FACETED / FILTERED - separate them with + or &amp;:   NATIONAL + COPPER   - and a lot lights up only if it matches EVERY facet.   •   the two mix:   OMKAR, STERLING + COPPER   = (OMKAR or STERLING) and COPPER.   Up to 8 values, empty ones ignored, spaces around a separator are fine.  •   THE RESULT IS GROUPED BY THE VALUE YOU TYPED: every value gets its own block of lots with a shaded ∑ total row beneath it, then a blue TOTAL MATCHED row adds every group up at once - the grand total of the rows your search actually hit, sitting right beneath them.  Under that a greyed REMAINING block holds the lots that did not match, with its own total, and the green GRAND TOTAL of both sits at the foot.  A lot matching two values is counted under the first one only, so TOTAL MATCHED + REMAINING always equals GRAND TOTAL, and with nothing typed the matched row is the whole list.   •   clear the box and all 37 come back in one ALL LOTS block.   •   cell F3 narrows what the text is looked for in (lot no. + buyer + name by default).   •   matching is contains, not case sensitive.   •   nothing here is typed in: every figure is a live link to Final Calculation Sheet.   •   columns AK..CU are hidden helpers.</t>
+    <t>HOW TO USE  ▶  click the yellow box B3 and type - a lot number (1874), part of one (187), a buyer (NATIONAL), part of a buyer name, a lot name (COPPER).   •   WILDCARD / MATCH ANY - separate values with a comma or a slash:   1874, 1923, OMKAR   or   1874 / 1923    - and every lot containing ANY of them lights up.   •   COLUMN SEARCHES - type above any column header in row 4; comma or slash means ANY value in that column, * matches any text and ? matches one character.  Filters entered in different columns are combined as ALL.   •   FACETED / FILTERED - separate them with + or &amp;:   NATIONAL + COPPER   - and a lot lights up only if it matches EVERY facet.   •   the two mix:   OMKAR, STERLING + COPPER   = (OMKAR or STERLING) and COPPER.   Up to 8 values, empty ones ignored, spaces around a separator are fine.  •   THE RESULT IS GROUPED BY THE VALUE YOU TYPED: every value gets its own block of lots with a shaded ∑ total row beneath it, then a blue TOTAL MATCHED row adds every group up at once - the grand total of the rows your search actually hit, sitting right beneath them.  Under that a greyed REMAINING block holds the lots that did not match, with its own total, and the green GRAND TOTAL of both sits at the foot.  A lot matching two values is counted under the first one only, so TOTAL MATCHED + REMAINING always equals GRAND TOTAL, and with nothing typed the matched row is the whole list.   •   clear the box and all 37 come back in one ALL LOTS block.   •   cell F3 narrows what the text is looked for in (lot no. + buyer + name by default).   •   matching is contains, not case sensitive.   •   nothing here is typed in: every figure is a live link to Final Calculation Sheet.   •   columns AK..CU are hidden helpers.   •   use the +/- outline control above columns D:H to expand/collapse Lot Name through Rate under Buyer.</t>
   </si>
   <si>
     <t>🔍  SEARCH  ▸</t>
@@ -6078,22 +6078,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
+    <outlinePr summaryRight="1" summaryBelow="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:CU54"/>
-  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="34" width="13.42578125" customWidth="1"/>
@@ -6101,7 +6102,7 @@
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99" ht="30" customHeight="1" ns3:dyDescent="0.25">
+    <row r="1" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="81" t="s">
         <v>122</v>
       </c>
@@ -6140,7 +6141,7 @@
       <c r="AH1" s="77"/>
       <c r="AI1" s="77"/>
     </row>
-    <row r="2" spans="1:99" ht="44.1" customHeight="1" ns3:dyDescent="0.25">
+    <row r="2" spans="1:99" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="76" t="s">
         <v>123</v>
       </c>
@@ -6179,7 +6180,7 @@
       <c r="AH2" s="77"/>
       <c r="AI2" s="77"/>
     </row>
-    <row r="3" spans="1:99" ht="30" customHeight="1" ns3:dyDescent="0.25">
+    <row r="3" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="59" t="s">
         <v>124</v>
       </c>
@@ -6247,7 +6248,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:99" ht="30" customHeight="1" ns3:dyDescent="0.25">
+    <row r="4" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="61"/>
       <c r="B4" s="61"/>
       <c r="C4" s="61"/>
@@ -6338,7 +6339,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:99" ht="44.1" customHeight="1" ns3:dyDescent="0.25">
+    <row r="5" spans="1:99" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
         <v>133</v>
       </c>
@@ -6679,7 +6680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="6" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="67">
         <f>IF($BJ5&gt;0,INDEX($BA$5:$BA$41,MATCH(5,$BB$5:$BB$41,0)),IF(OR($BI5=1,$BL5=1,$BH5&gt;0),"∑",""))</f>
         <v>1</v>
@@ -7051,7 +7052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="7" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="67">
         <f>IF($BJ6&gt;0,INDEX($BA$5:$BA$41,MATCH(6,$BB$5:$BB$41,0)),IF(OR($BI6=1,$BL6=1,$BH6&gt;0),"∑",""))</f>
         <v>2</v>
@@ -7423,7 +7424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="8" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="67">
         <f>IF($BJ7&gt;0,INDEX($BA$5:$BA$41,MATCH(7,$BB$5:$BB$41,0)),IF(OR($BI7=1,$BL7=1,$BH7&gt;0),"∑",""))</f>
         <v>3</v>
@@ -7794,7 +7795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="9" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="67">
         <f>IF($BJ8&gt;0,INDEX($BA$5:$BA$41,MATCH(8,$BB$5:$BB$41,0)),IF(OR($BI8=1,$BL8=1,$BH8&gt;0),"∑",""))</f>
         <v>4</v>
@@ -8166,7 +8167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="10" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="67" t="str">
         <f>IF($BJ9&gt;0,INDEX($BA$5:$BA$41,MATCH(9,$BB$5:$BB$41,0)),IF(OR($BI9=1,$BL9=1,$BH9&gt;0),"∑",""))</f>
         <v>∑</v>
@@ -8503,7 +8504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="11" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="67">
         <f>IF($BJ10&gt;0,INDEX($BA$5:$BA$41,MATCH(10,$BB$5:$BB$41,0)),IF(OR($BI10=1,$BL10=1,$BH10&gt;0),"∑",""))</f>
         <v>1</v>
@@ -8840,7 +8841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="12" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="67">
         <f>IF($BJ11&gt;0,INDEX($BA$5:$BA$41,MATCH(11,$BB$5:$BB$41,0)),IF(OR($BI11=1,$BL11=1,$BH11&gt;0),"∑",""))</f>
         <v>2</v>
@@ -9177,7 +9178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="13" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="67">
         <f>IF($BJ12&gt;0,INDEX($BA$5:$BA$41,MATCH(12,$BB$5:$BB$41,0)),IF(OR($BI12=1,$BL12=1,$BH12&gt;0),"∑",""))</f>
         <v>3</v>
@@ -9514,7 +9515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="14" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="67">
         <f>IF($BJ13&gt;0,INDEX($BA$5:$BA$41,MATCH(13,$BB$5:$BB$41,0)),IF(OR($BI13=1,$BL13=1,$BH13&gt;0),"∑",""))</f>
         <v>4</v>
@@ -9839,7 +9840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="15" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="67">
         <f>IF($BJ14&gt;0,INDEX($BA$5:$BA$41,MATCH(14,$BB$5:$BB$41,0)),IF(OR($BI14=1,$BL14=1,$BH14&gt;0),"∑",""))</f>
         <v>5</v>
@@ -10164,7 +10165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="16" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="67" t="str">
         <f>IF($BJ15&gt;0,INDEX($BA$5:$BA$41,MATCH(15,$BB$5:$BB$41,0)),IF(OR($BI15=1,$BL15=1,$BH15&gt;0),"∑",""))</f>
         <v>∑</v>
@@ -10489,7 +10490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="17" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="str">
         <f>IF($BJ16&gt;0,INDEX($BA$5:$BA$41,MATCH(16,$BB$5:$BB$41,0)),IF(OR($BI16=1,$BL16=1,$BH16&gt;0),"∑",""))</f>
         <v>∑</v>
@@ -10814,7 +10815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="18" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="67">
         <f>IF($BJ17&gt;0,INDEX($BA$5:$BA$41,MATCH(17,$BB$5:$BB$41,0)),IF(OR($BI17=1,$BL17=1,$BH17&gt;0),"∑",""))</f>
         <v>1</v>
@@ -11139,7 +11140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="19" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="67">
         <f>IF($BJ18&gt;0,INDEX($BA$5:$BA$41,MATCH(18,$BB$5:$BB$41,0)),IF(OR($BI18=1,$BL18=1,$BH18&gt;0),"∑",""))</f>
         <v>2</v>
@@ -11464,7 +11465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="20" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="67">
         <f>IF($BJ19&gt;0,INDEX($BA$5:$BA$41,MATCH(19,$BB$5:$BB$41,0)),IF(OR($BI19=1,$BL19=1,$BH19&gt;0),"∑",""))</f>
         <v>3</v>
@@ -11789,7 +11790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="21" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="67">
         <f>IF($BJ20&gt;0,INDEX($BA$5:$BA$41,MATCH(20,$BB$5:$BB$41,0)),IF(OR($BI20=1,$BL20=1,$BH20&gt;0),"∑",""))</f>
         <v>4</v>
@@ -12114,7 +12115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="22" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="67">
         <f>IF($BJ21&gt;0,INDEX($BA$5:$BA$41,MATCH(21,$BB$5:$BB$41,0)),IF(OR($BI21=1,$BL21=1,$BH21&gt;0),"∑",""))</f>
         <v>5</v>
@@ -12439,7 +12440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="23" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="67">
         <f>IF($BJ22&gt;0,INDEX($BA$5:$BA$41,MATCH(22,$BB$5:$BB$41,0)),IF(OR($BI22=1,$BL22=1,$BH22&gt;0),"∑",""))</f>
         <v>6</v>
@@ -12764,7 +12765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="24" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="67">
         <f>IF($BJ23&gt;0,INDEX($BA$5:$BA$41,MATCH(23,$BB$5:$BB$41,0)),IF(OR($BI23=1,$BL23=1,$BH23&gt;0),"∑",""))</f>
         <v>7</v>
@@ -13089,7 +13090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="25" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="67">
         <f>IF($BJ24&gt;0,INDEX($BA$5:$BA$41,MATCH(24,$BB$5:$BB$41,0)),IF(OR($BI24=1,$BL24=1,$BH24&gt;0),"∑",""))</f>
         <v>8</v>
@@ -13414,7 +13415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="26" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="67">
         <f>IF($BJ25&gt;0,INDEX($BA$5:$BA$41,MATCH(25,$BB$5:$BB$41,0)),IF(OR($BI25=1,$BL25=1,$BH25&gt;0),"∑",""))</f>
         <v>9</v>
@@ -13739,7 +13740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="27" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="67">
         <f>IF($BJ26&gt;0,INDEX($BA$5:$BA$41,MATCH(26,$BB$5:$BB$41,0)),IF(OR($BI26=1,$BL26=1,$BH26&gt;0),"∑",""))</f>
         <v>10</v>
@@ -14064,7 +14065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="28" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="67">
         <f>IF($BJ27&gt;0,INDEX($BA$5:$BA$41,MATCH(27,$BB$5:$BB$41,0)),IF(OR($BI27=1,$BL27=1,$BH27&gt;0),"∑",""))</f>
         <v>11</v>
@@ -14389,7 +14390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="29" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="67">
         <f>IF($BJ28&gt;0,INDEX($BA$5:$BA$41,MATCH(28,$BB$5:$BB$41,0)),IF(OR($BI28=1,$BL28=1,$BH28&gt;0),"∑",""))</f>
         <v>12</v>
@@ -14714,7 +14715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="30" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="67">
         <f>IF($BJ29&gt;0,INDEX($BA$5:$BA$41,MATCH(29,$BB$5:$BB$41,0)),IF(OR($BI29=1,$BL29=1,$BH29&gt;0),"∑",""))</f>
         <v>13</v>
@@ -15039,7 +15040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="31" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="67">
         <f>IF($BJ30&gt;0,INDEX($BA$5:$BA$41,MATCH(30,$BB$5:$BB$41,0)),IF(OR($BI30=1,$BL30=1,$BH30&gt;0),"∑",""))</f>
         <v>14</v>
@@ -15364,7 +15365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="32" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="67">
         <f>IF($BJ31&gt;0,INDEX($BA$5:$BA$41,MATCH(31,$BB$5:$BB$41,0)),IF(OR($BI31=1,$BL31=1,$BH31&gt;0),"∑",""))</f>
         <v>15</v>
@@ -15689,7 +15690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="33" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="67">
         <f>IF($BJ32&gt;0,INDEX($BA$5:$BA$41,MATCH(32,$BB$5:$BB$41,0)),IF(OR($BI32=1,$BL32=1,$BH32&gt;0),"∑",""))</f>
         <v>16</v>
@@ -16014,7 +16015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="34" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="67">
         <f>IF($BJ33&gt;0,INDEX($BA$5:$BA$41,MATCH(33,$BB$5:$BB$41,0)),IF(OR($BI33=1,$BL33=1,$BH33&gt;0),"∑",""))</f>
         <v>17</v>
@@ -16339,7 +16340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="35" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="67">
         <f>IF($BJ34&gt;0,INDEX($BA$5:$BA$41,MATCH(34,$BB$5:$BB$41,0)),IF(OR($BI34=1,$BL34=1,$BH34&gt;0),"∑",""))</f>
         <v>18</v>
@@ -16664,7 +16665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="36" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="67">
         <f>IF($BJ35&gt;0,INDEX($BA$5:$BA$41,MATCH(35,$BB$5:$BB$41,0)),IF(OR($BI35=1,$BL35=1,$BH35&gt;0),"∑",""))</f>
         <v>19</v>
@@ -16989,7 +16990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="37" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="67">
         <f>IF($BJ36&gt;0,INDEX($BA$5:$BA$41,MATCH(36,$BB$5:$BB$41,0)),IF(OR($BI36=1,$BL36=1,$BH36&gt;0),"∑",""))</f>
         <v>20</v>
@@ -17314,7 +17315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="38" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="67">
         <f>IF($BJ37&gt;0,INDEX($BA$5:$BA$41,MATCH(37,$BB$5:$BB$41,0)),IF(OR($BI37=1,$BL37=1,$BH37&gt;0),"∑",""))</f>
         <v>21</v>
@@ -17639,7 +17640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="39" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="67">
         <f>IF($BJ38&gt;0,INDEX($BA$5:$BA$41,MATCH(38,$BB$5:$BB$41,0)),IF(OR($BI38=1,$BL38=1,$BH38&gt;0),"∑",""))</f>
         <v>22</v>
@@ -17964,7 +17965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="40" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="67">
         <f>IF($BJ39&gt;0,INDEX($BA$5:$BA$41,MATCH(39,$BB$5:$BB$41,0)),IF(OR($BI39=1,$BL39=1,$BH39&gt;0),"∑",""))</f>
         <v>23</v>
@@ -18289,7 +18290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="41" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="67">
         <f>IF($BJ40&gt;0,INDEX($BA$5:$BA$41,MATCH(40,$BB$5:$BB$41,0)),IF(OR($BI40=1,$BL40=1,$BH40&gt;0),"∑",""))</f>
         <v>24</v>
@@ -18614,7 +18615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="42" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="67">
         <f>IF($BJ41&gt;0,INDEX($BA$5:$BA$41,MATCH(41,$BB$5:$BB$41,0)),IF(OR($BI41=1,$BL41=1,$BH41&gt;0),"∑",""))</f>
         <v>25</v>
@@ -18776,7 +18777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="43" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="67">
         <f>IF($BJ42&gt;0,INDEX($BA$5:$BA$41,MATCH(42,$BB$5:$BB$41,0)),IF(OR($BI42=1,$BL42=1,$BH42&gt;0),"∑",""))</f>
         <v>26</v>
@@ -18938,7 +18939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="44" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="67">
         <f>IF($BJ43&gt;0,INDEX($BA$5:$BA$41,MATCH(43,$BB$5:$BB$41,0)),IF(OR($BI43=1,$BL43=1,$BH43&gt;0),"∑",""))</f>
         <v>27</v>
@@ -19100,7 +19101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="45" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="67">
         <f>IF($BJ44&gt;0,INDEX($BA$5:$BA$41,MATCH(44,$BB$5:$BB$41,0)),IF(OR($BI44=1,$BL44=1,$BH44&gt;0),"∑",""))</f>
         <v>28</v>
@@ -19262,7 +19263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="46" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="67" t="str">
         <f>IF($BJ45&gt;0,INDEX($BA$5:$BA$41,MATCH(45,$BB$5:$BB$41,0)),IF(OR($BI45=1,$BL45=1,$BH45&gt;0),"∑",""))</f>
         <v>∑</v>
@@ -19424,7 +19425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="47" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="67" t="str">
         <f>IF($BJ46&gt;0,INDEX($BA$5:$BA$41,MATCH(46,$BB$5:$BB$41,0)),IF(OR($BI46=1,$BL46=1,$BH46&gt;0),"∑",""))</f>
         <v>∑</v>
@@ -19586,7 +19587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="48" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="67" t="str">
         <f>IF($BJ47&gt;0,INDEX($BA$5:$BA$41,MATCH(47,$BB$5:$BB$41,0)),IF(OR($BI47=1,$BL47=1,$BH47&gt;0),"∑",""))</f>
         <v/>
@@ -19748,7 +19749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="49" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="67" t="str">
         <f>IF($BJ48&gt;0,INDEX($BA$5:$BA$41,MATCH(48,$BB$5:$BB$41,0)),IF(OR($BI48=1,$BL48=1,$BH48&gt;0),"∑",""))</f>
         <v/>
@@ -19910,7 +19911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="50" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="67" t="str">
         <f>IF($BJ49&gt;0,INDEX($BA$5:$BA$41,MATCH(49,$BB$5:$BB$41,0)),IF(OR($BI49=1,$BL49=1,$BH49&gt;0),"∑",""))</f>
         <v/>
@@ -20072,7 +20073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="51" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="67" t="str">
         <f>IF($BJ50&gt;0,INDEX($BA$5:$BA$41,MATCH(50,$BB$5:$BB$41,0)),IF(OR($BI50=1,$BL50=1,$BH50&gt;0),"∑",""))</f>
         <v/>
@@ -20234,7 +20235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="52" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="67" t="str">
         <f>IF($BJ51&gt;0,INDEX($BA$5:$BA$41,MATCH(51,$BB$5:$BB$41,0)),IF(OR($BI51=1,$BL51=1,$BH51&gt;0),"∑",""))</f>
         <v/>
@@ -20396,7 +20397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="53" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="67" t="str">
         <f>IF($BJ52&gt;0,INDEX($BA$5:$BA$41,MATCH(52,$BB$5:$BB$41,0)),IF(OR($BI52=1,$BL52=1,$BH52&gt;0),"∑",""))</f>
         <v/>
@@ -20558,7 +20559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:99" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="54" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="67" t="str">
         <f>IF($BJ53&gt;0,INDEX($BA$5:$BA$41,MATCH(53,$BB$5:$BB$41,0)),IF(OR($BI53=1,$BL53=1,$BH53&gt;0),"∑",""))</f>
         <v/>
@@ -20749,7 +20750,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="F3" ns2:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" sqref="F3" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>$AO$4:$AO$9</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="A4:AI4" promptTitle="Column wildcard search" prompt="Type text; comma or / means ANY. Use * for any text or ? for one character.">

</xml_diff>

<commit_message>
Fix workbook namespace declarations
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20361"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <ns2:absPath url="C:\Users\S.M.C\Downloads\"/>
+      <x15ac:absPath url="C:\Users\S.M.C\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D8CAA5-FA05-4AFF-A696-DFAD20822EA2}" ns4:coauthVersionLast="36" ns4:coauthVersionMax="36" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D8CAA5-FA05-4AFF-A696-DFAD20822EA2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11385" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6078,7 +6078,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <outlinePr summaryRight="1" summaryBelow="1"/>

</xml_diff>

<commit_message>
Group GST columns under material value
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -6096,8 +6096,9 @@
     <col min="7" max="7" width="11" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="34" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="34" width="13.42578125" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Group GST TDS rate under GST TDS
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -6100,7 +6100,9 @@
     <col min="11" max="11" width="13.42578125" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="13.42578125" customWidth="1" outlineLevel="1"/>
     <col min="13" max="16" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="17" max="34" width="13.42578125" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="19" max="34" width="13.42578125" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Group security deposit received column
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -6102,7 +6102,9 @@
     <col min="13" max="16" width="13.42578125" customWidth="1" outlineLevel="1"/>
     <col min="17" max="17" width="13.42578125" customWidth="1"/>
     <col min="18" max="18" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="19" max="34" width="13.42578125" customWidth="1"/>
+    <col min="19" max="20" width="13.42578125" customWidth="1"/>
+    <col min="21" max="21" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="34" width="13.42578125" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Group final payment received column
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -6104,7 +6104,9 @@
     <col min="18" max="18" width="13.42578125" customWidth="1" outlineLevel="1"/>
     <col min="19" max="20" width="13.42578125" customWidth="1"/>
     <col min="21" max="21" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="34" width="13.42578125" customWidth="1"/>
+    <col min="22" max="23" width="13.42578125" customWidth="1"/>
+    <col min="24" max="24" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="34" width="13.42578125" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Group LPP expected column
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/07.09.2026.xlsx
+++ b/07.09.2026.xlsx
@@ -6106,7 +6106,9 @@
     <col min="21" max="21" width="13.42578125" customWidth="1" outlineLevel="1"/>
     <col min="22" max="23" width="13.42578125" customWidth="1"/>
     <col min="24" max="24" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="34" width="13.42578125" customWidth="1"/>
+    <col min="25" max="26" width="13.42578125" customWidth="1"/>
+    <col min="27" max="27" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="34" width="13.42578125" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
     <col min="37" max="99" width="12" hidden="1" customWidth="1"/>
   </cols>

</xml_diff>